<commit_message>
chore(daily): 自动更新 data.js + stock_data.xlsx (北京时间 2026-10-21 03:48)
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20799,6 +20799,48 @@
       </c>
       <c r="L485" t="n">
         <v>-0.01179498177139193</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="D486" t="n">
+        <v>47.45</v>
+      </c>
+      <c r="E486" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="F486" t="n">
+        <v>47.45</v>
+      </c>
+      <c r="G486" t="n">
+        <v>46.08</v>
+      </c>
+      <c r="H486" t="n">
+        <v>1.370000000000005</v>
+      </c>
+      <c r="I486" t="n">
+        <v>2.973090277777788</v>
+      </c>
+      <c r="J486" t="n">
+        <v>72076406</v>
+      </c>
+      <c r="K486" t="n">
+        <v>3371373900</v>
+      </c>
+      <c r="L486" t="n">
+        <v>0.0297309027777779</v>
       </c>
     </row>
   </sheetData>
@@ -20812,7 +20854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41199,6 +41241,48 @@
       </c>
       <c r="L485" t="n">
         <v>-0.01179498177139193</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="D486" t="n">
+        <v>47.45</v>
+      </c>
+      <c r="E486" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="F486" t="n">
+        <v>47.45</v>
+      </c>
+      <c r="G486" t="n">
+        <v>46.08</v>
+      </c>
+      <c r="H486" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="I486" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="J486" t="n">
+        <v>719586</v>
+      </c>
+      <c r="K486" t="n">
+        <v>3371373924</v>
+      </c>
+      <c r="L486" t="n">
+        <v>0.0297309027777779</v>
       </c>
     </row>
   </sheetData>
@@ -41212,7 +41296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61595,6 +61679,48 @@
       </c>
       <c r="L485" t="n">
         <v>0.01304347826086949</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="D486" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="F486" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="G486" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.2100000000000009</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-1.802575107296144</v>
+      </c>
+      <c r="J486" t="n">
+        <v>123986114</v>
+      </c>
+      <c r="K486" t="n">
+        <v>1429559900</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.01802575107296145</v>
       </c>
     </row>
   </sheetData>
@@ -61608,7 +61734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81993,6 +82119,48 @@
         <v>0.01304347826086949</v>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="D486" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="F486" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="G486" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.2100000000000009</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-1.802575107296144</v>
+      </c>
+      <c r="J486" t="n">
+        <v>123986114</v>
+      </c>
+      <c r="K486" t="n">
+        <v>1429559900</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.01802575107296145</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(daily): 自动更新 data.js + stock_data.xlsx (北京时间 2026-10-29 04:44)
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20841,6 +20841,48 @@
       </c>
       <c r="L486" t="n">
         <v>-0.03085106382978731</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>47</v>
+      </c>
+      <c r="D487" t="n">
+        <v>49.22</v>
+      </c>
+      <c r="E487" t="n">
+        <v>46.68</v>
+      </c>
+      <c r="F487" t="n">
+        <v>48.36</v>
+      </c>
+      <c r="G487" t="n">
+        <v>45.55</v>
+      </c>
+      <c r="H487" t="n">
+        <v>2.810000000000002</v>
+      </c>
+      <c r="I487" t="n">
+        <v>6.16904500548848</v>
+      </c>
+      <c r="J487" t="n">
+        <v>151810847</v>
+      </c>
+      <c r="K487" t="n">
+        <v>7238341200</v>
+      </c>
+      <c r="L487" t="n">
+        <v>0.06169045005488472</v>
       </c>
     </row>
   </sheetData>
@@ -20854,7 +20896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41279,6 +41321,48 @@
       </c>
       <c r="L486" t="n">
         <v>-0.03085106382978731</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>47</v>
+      </c>
+      <c r="D487" t="n">
+        <v>49.22</v>
+      </c>
+      <c r="E487" t="n">
+        <v>46.68</v>
+      </c>
+      <c r="F487" t="n">
+        <v>48.36</v>
+      </c>
+      <c r="G487" t="n">
+        <v>45.55</v>
+      </c>
+      <c r="H487" t="n">
+        <v>2.810000000000002</v>
+      </c>
+      <c r="I487" t="n">
+        <v>6.16904500548848</v>
+      </c>
+      <c r="J487" t="n">
+        <v>151810847</v>
+      </c>
+      <c r="K487" t="n">
+        <v>7238341200</v>
+      </c>
+      <c r="L487" t="n">
+        <v>0.06169045005488472</v>
       </c>
     </row>
   </sheetData>
@@ -41292,7 +41376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61717,6 +61801,48 @@
       </c>
       <c r="L486" t="n">
         <v>0.01504424778761071</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="D487" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E487" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="F487" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="G487" t="n">
+        <v>11.47</v>
+      </c>
+      <c r="H487" t="n">
+        <v>-0.1600000000000001</v>
+      </c>
+      <c r="I487" t="n">
+        <v>-1.394943330427203</v>
+      </c>
+      <c r="J487" t="n">
+        <v>168122058</v>
+      </c>
+      <c r="K487" t="n">
+        <v>1911547800</v>
+      </c>
+      <c r="L487" t="n">
+        <v>-0.01394943330427201</v>
       </c>
     </row>
   </sheetData>
@@ -61730,7 +61856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82157,6 +82283,48 @@
         <v>0.01504424778761071</v>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="D487" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E487" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="F487" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="G487" t="n">
+        <v>11.47</v>
+      </c>
+      <c r="H487" t="n">
+        <v>-0.1600000000000001</v>
+      </c>
+      <c r="I487" t="n">
+        <v>-1.394943330427203</v>
+      </c>
+      <c r="J487" t="n">
+        <v>168122058</v>
+      </c>
+      <c r="K487" t="n">
+        <v>1911547800</v>
+      </c>
+      <c r="L487" t="n">
+        <v>-0.01394943330427201</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>